<commit_message>
Update input Excel db_plano_corte.xlsx
Replace the files/input/db_plano_corte.xlsx binary with an updated version. This commit updates the Excel spreadsheet contents (data or formatting changes) used as input for the project.
</commit_message>
<xml_diff>
--- a/files/input/db_plano_corte.xlsx
+++ b/files/input/db_plano_corte.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acotelcombr-my.sharepoint.com/personal/jefersson_souza_acotel_com_br/Documents/Dev/Plano_corte_py/files/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\#Mega\Jeferson - Dev\02 - Linguagens\Python\Acotel\Plano_corte_sliter_py\files\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="244" documentId="11_D5931D32DBA823BFB85A9752573287776C05D6AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10434D4B-0879-42C0-82B7-641E371E72D1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C8EC4D-0AA6-46B8-B84A-32DF8E6CEFD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="810" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -5169,16 +5169,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -5312,7 +5303,7 @@
     <col min="6" max="6" width="18.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.7109375" style="1" customWidth="1"/>
     <col min="10" max="16384" width="11.5703125" style="1"/>
   </cols>
   <sheetData>

</xml_diff>